<commit_message>
Package final password security results
</commit_message>
<xml_diff>
--- a/PasswordSecurity/results/final/Password-Security-Final.xlsx
+++ b/PasswordSecurity/results/final/Password-Security-Final.xlsx
@@ -1,16 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Measured Time" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Search Space" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measured Time" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search Space" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Science Buddies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -241,13 +243,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -271,10 +273,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2563EB"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -302,8 +304,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -330,8 +332,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -354,13 +356,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -383,7 +385,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="2563EB"/>
               </a:solidFill>
@@ -393,7 +395,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -418,7 +420,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="16A34A"/>
               </a:solidFill>
@@ -428,7 +430,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -453,7 +455,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="DC2626"/>
               </a:solidFill>
@@ -463,7 +465,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -488,7 +490,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="9333EA"/>
               </a:solidFill>
@@ -498,7 +500,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -526,8 +528,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -554,8 +556,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -581,13 +583,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -610,7 +612,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="2563EB"/>
               </a:solidFill>
@@ -620,7 +622,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -645,7 +647,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="16A34A"/>
               </a:solidFill>
@@ -655,7 +657,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -680,7 +682,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="DC2626"/>
               </a:solidFill>
@@ -690,7 +692,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -715,7 +717,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="26000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="26000">
               <a:solidFill>
                 <a:srgbClr val="9333EA"/>
               </a:solidFill>
@@ -725,7 +727,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -753,8 +755,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -781,8 +783,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -808,7 +810,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -823,9 +825,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -835,7 +837,7 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -850,9 +852,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -862,7 +864,7 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -877,9 +879,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -937,6 +939,31 @@
   <tableColumns count="2">
     <tableColumn id="1" name="Topic"/>
     <tableColumn id="2" name="Explanation"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ScienceBuddiesChecklist" displayName="ScienceBuddiesChecklist" ref="A4:C13" headerRowCount="1">
+  <autoFilter ref="A4:C13"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Requested work"/>
+    <tableColumn id="2" name="What this project did"/>
+    <tableColumn id="3" name="Evidence"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PasswordResearchNotes" displayName="PasswordResearchNotes" ref="A4:D16" headerRowCount="1">
+  <autoFilter ref="A4:D16"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Topic"/>
+    <tableColumn id="2" name="Research note"/>
+    <tableColumn id="3" name="Connection to this experiment"/>
+    <tableColumn id="4" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1232,7 +1259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1485,23 +1512,22 @@
         <v>29263</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Conclusion: Challenge 6 was not a six-character password made only from A–Z, a–z, and 0–9. This rules out only that tested search space.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38"/>
+          <t>We tested every six-character password made from A-Z, a-z, and 0-9, but none matched Challenge 6. It must be outside that tested search space.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="E4:F6"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A37:H38"/>
     <mergeCell ref="C4:D6"/>
     <mergeCell ref="A4:B6"/>
     <mergeCell ref="G4:H6"/>
+    <mergeCell ref="A37:H37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2015,4 +2041,543 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="0016A34A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SCIENCE BUDDIES CHECKLIST</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>How the completed project answers the assigned procedure</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Requested work</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>What this project did</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Research password strength</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Compared length, character-set size, predictability, and guessing strategy.</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Research Notes and final report</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Calculate combinations</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Calculated A^L for four alphabets and lengths 1–8.</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Search Space tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Graph exponential growth</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Created logarithmic graphs because the counts span many orders of magnitude.</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Search Space tab and graph files</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Write a guessing program</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Implemented the experiment in C# and retained the supplied Python files with attribution.</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Program.cs, Challenges.cs, and original/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Compare algorithms</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Measured numeric brute force, alphanumeric brute force, dictionary guesses, and word-pair guesses.</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Overview and challenge-summary.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Test supplied challenges</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Recovered Challenges 0–5 and fully tested one defined search space for Challenge 6.</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Overview and CHALLENGE-RESULTS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Record time and guesses</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Recorded attempt counts, elapsed time, repeated trials, and throughput.</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Measured Time and Overview tabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Use authorized samples</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Used Science Buddies samples and synthetic benchmarks; no real accounts or private passwords.</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Notes tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Credit starter material</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>Science Buddies files remain in original/ with their attribution.</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sciencebuddies.org/science-fair-projects/project-ideas/CompSci_p046/computer-science/password-security-how-easily-can-your-password-be-hacked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="009333EA"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PASSWORD SECURITY RESEARCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Background needed to interpret the classroom experiment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Research note</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Connection to this experiment</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="68" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Search space</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>For an alphabet of A characters and fixed length L, brute force has A^L candidates.</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Adding one character multiplies worst-case work by A.</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sciencebuddies.org/science-fair-projects/project-ideas/CompSci_p046/computer-science/password-security-how-easily-can-your-password-be-hacked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="68" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Dictionary attacks</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>People often choose predictable words and patterns, so likely guesses can beat exhaustive brute force.</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>The dictionary recovered two challenges in fewer than 500 guesses.</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sciencebuddies.org/science-fair-projects/project-ideas/CompSci_p046/computer-science/password-security-how-easily-can-your-password-be-hacked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="68" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Word combinations</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Combining familiar words can remain predictable when an attacker tests word pairs.</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>The experiment recovered secretpassword with the word-pair method.</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sciencebuddies.org/science-fair-projects/project-ideas/CompSci_p046/computer-science/password-security-how-easily-can-your-password-be-hacked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="68" customHeight="1">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>Password length</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Current NIST guidance treats length as a primary strength factor and supports long passphrases.</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>The search-space graph shows why every extra character matters.</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>https://pages.nist.gov/800-63-4/sp800-63b.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Blocklists</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>NIST requires services to reject commonly used, expected, or compromised passwords.</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Values such as 123 and dictionary words should be rejected even if they meet format rules.</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>https://pages.nist.gov/800-63-4/sp800-63b.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Composition rules</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>NIST says services should not force mixtures of character types because people respond predictably.</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>A capital letter or symbol does not automatically make a password unpredictable.</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>https://pages.nist.gov/800-63-4/sp800-63b.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="68" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Rate limiting</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Online services should limit failed authentication attempts.</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>This experiment modeled offline guessing; real online attempts should be restricted.</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>https://pages.nist.gov/800-63-4/sp800-63b.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>Hashing</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Hashing supports one-way verification, while encryption is reversible with a key.</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>The program compared MD5 outputs; it did not decrypt passwords.</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>https://cheatsheetseries.owasp.org/cheatsheets/Password_Storage_Cheat_Sheet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Salts</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>A unique random salt prevents one precomputed table from working against many password hashes.</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>The Science Buddies MD5 samples were unsalted and simpler than modern storage.</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>https://cheatsheetseries.owasp.org/cheatsheets/Password_Storage_Cheat_Sheet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="68" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Slow password hashing</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>OWASP recommends purpose-built algorithms such as Argon2id instead of fast general hashes.</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>The measured speed shows why fast MD5 is unsuitable for password storage.</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>https://cheatsheetseries.owasp.org/cheatsheets/Password_Storage_Cheat_Sheet.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Experiment limit</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>A failed search proves only that its defined candidate set did not contain a match.</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Challenge 6 may use another length, symbols, spaces, or a different pattern.</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Experimental result</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="68" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Ethics</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Password testing must be limited to systems and samples with explicit authorization.</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Only classroom data and synthetic passwords were tested.</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>https://www.sciencebuddies.org/science-fair-projects/project-ideas/CompSci_p046/computer-science/password-security-how-easily-can-your-password-be-hacked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>